<commit_message>
Auto stash before merge of "master" and "origin/master"
</commit_message>
<xml_diff>
--- a/xls2rdf-lib/src/test/resources/excel/suite/_01_exemple1/input.xlsx
+++ b/xls2rdf-lib/src/test/resources/excel/suite/_01_exemple1/input.xlsx
@@ -1,42 +1,53 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="120" windowWidth="27135" windowHeight="11955" activeTab="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
-    <sheet name="Feuil2" sheetId="2" r:id="rId2"/>
-    <sheet name="Feuil3" sheetId="3" r:id="rId3"/>
+    <sheet name="Feuil1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Feuil2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Feuil3" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
-    <t>dct:title</t>
+    <t xml:space="preserve">ConceptScheme URI</t>
+  </si>
+  <si>
+    <t>http://data.sparna.fr/vocabularies/days</t>
+  </si>
+  <si>
+    <t>dct:title@fr</t>
   </si>
   <si>
     <t>Weekdays</t>
   </si>
   <si>
-    <t>dct:description</t>
-  </si>
-  <si>
-    <t>The days of the week</t>
+    <t>dct:description@fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The days of the week</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This is a general comment that will be ignored. The converter will detect automatically the line containing the column titles below, so you can have a header as long as you want.</t>
   </si>
   <si>
     <t>URI</t>
   </si>
   <si>
-    <t>skos:prefLabel</t>
-  </si>
-  <si>
-    <t>skos:definition</t>
+    <t>skos:prefLabel@fr</t>
+  </si>
+  <si>
+    <t>skos:definition@fr</t>
   </si>
   <si>
     <t>skos:narrower</t>
@@ -45,123 +56,112 @@
     <t>skos:notation</t>
   </si>
   <si>
+    <t>http://data.sparna.fr/vocabularies/days#monday</t>
+  </si>
+  <si>
     <t>Monday</t>
   </si>
   <si>
-    <t>The day where you get back at work</t>
+    <t xml:space="preserve">The day where you get back at work</t>
   </si>
   <si>
     <t>MON</t>
   </si>
   <si>
+    <t>http://data.sparna.fr/vocabularies/days#tuesday</t>
+  </si>
+  <si>
     <t>Tuesday</t>
   </si>
   <si>
-    <t>The most productive day of the week.</t>
+    <t xml:space="preserve">The most productive day of the week.</t>
   </si>
   <si>
     <t>TUE</t>
   </si>
   <si>
+    <t>http://data.sparna.fr/vocabularies/days#wednesday</t>
+  </si>
+  <si>
     <t>Wednesday</t>
   </si>
   <si>
     <t>WED</t>
   </si>
   <si>
+    <t>http://data.sparna.fr/vocabularies/days#thursday</t>
+  </si>
+  <si>
     <t>Thursday</t>
   </si>
   <si>
     <t>THU</t>
   </si>
   <si>
+    <t>http://data.sparna.fr/vocabularies/days#friday</t>
+  </si>
+  <si>
     <t>Friday</t>
   </si>
   <si>
-    <t>Week-end soon !</t>
+    <t xml:space="preserve">Week-end soon !</t>
   </si>
   <si>
     <t>FRI</t>
   </si>
   <si>
+    <t>http://data.sparna.fr/vocabularies/days#saturday</t>
+  </si>
+  <si>
     <t>Saturday</t>
   </si>
   <si>
     <t>SAT</t>
   </si>
   <si>
+    <t>http://data.sparna.fr/vocabularies/days#sunday</t>
+  </si>
+  <si>
     <t>Sunday</t>
   </si>
   <si>
-    <t>The day you sleep.</t>
+    <t xml:space="preserve">The day you sleep.</t>
   </si>
   <si>
     <t>SUN</t>
   </si>
   <si>
+    <t>http://data.sparna.fr/vocabularies/days#week-end</t>
+  </si>
+  <si>
     <t>Week-end</t>
   </si>
   <si>
-    <t>Any day of the week-end</t>
+    <t xml:space="preserve">Any day of the week-end</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://data.sparna.fr/vocabularies/days#saturday, http://data.sparna.fr/vocabularies/days#sunday</t>
   </si>
   <si>
     <t>WKND</t>
-  </si>
-  <si>
-    <t>This is a general comment that will be ignored. The converter will detect automatically the line containing the column titles below, so you can have a header as long as you want.</t>
-  </si>
-  <si>
-    <t>http://data.sparna.fr/vocabularies/days</t>
-  </si>
-  <si>
-    <t>http://data.sparna.fr/vocabularies/days#monday</t>
-  </si>
-  <si>
-    <t>http://data.sparna.fr/vocabularies/days#tuesday</t>
-  </si>
-  <si>
-    <t>http://data.sparna.fr/vocabularies/days#wednesday</t>
-  </si>
-  <si>
-    <t>http://data.sparna.fr/vocabularies/days#thursday</t>
-  </si>
-  <si>
-    <t>http://data.sparna.fr/vocabularies/days#friday</t>
-  </si>
-  <si>
-    <t>http://data.sparna.fr/vocabularies/days#saturday</t>
-  </si>
-  <si>
-    <t>http://data.sparna.fr/vocabularies/days#sunday</t>
-  </si>
-  <si>
-    <t>http://data.sparna.fr/vocabularies/days#week-end</t>
-  </si>
-  <si>
-    <t>http://data.sparna.fr/vocabularies/days#saturday, http://data.sparna.fr/vocabularies/days#sunday</t>
-  </si>
-  <si>
-    <t>ConceptScheme URI</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="2">
     <font>
-      <sz val="11"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -175,46 +175,50 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
   <borders count="1">
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
   <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="1" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf fontId="1" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -259,13 +263,13 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Thai" typeface="Angsana New"/>
         <a:font script="Ethi" typeface="Nyala"/>
         <a:font script="Beng" typeface="Vrinda"/>
         <a:font script="Gujr" typeface="Shruti"/>
@@ -293,13 +297,13 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Thai" typeface="Cordia New"/>
         <a:font script="Ethi" typeface="Nyala"/>
         <a:font script="Beng" typeface="Vrinda"/>
         <a:font script="Gujr" typeface="Shruti"/>
@@ -496,196 +500,421 @@
 </a:theme>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Thème Office">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="50.28515625" customWidth="1"/>
-    <col min="2" max="2" width="36.42578125" customWidth="1"/>
-    <col min="3" max="3" width="26.7109375" customWidth="1"/>
-    <col min="4" max="4" width="45.7109375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="35.85546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="30.42578125" customWidth="1"/>
+    <col customWidth="1" min="1" max="1" width="50.28515625"/>
+    <col customWidth="1" min="2" max="2" width="36.42578125"/>
+    <col customWidth="1" min="3" max="3" width="26.7109375"/>
+    <col customWidth="1" min="4" max="4" style="1" width="45.7109375"/>
+    <col customWidth="1" min="5" max="5" style="1" width="35.85546875"/>
+    <col customWidth="1" min="6" max="6" width="30.42578125"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="5" t="s">
-        <v>41</v>
+    <row r="1">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" s="5" t="s">
-        <v>0</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C2" s="1"/>
     </row>
-    <row r="3" spans="1:5">
-      <c r="A3" s="5" t="s">
-        <v>2</v>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C3" s="1"/>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5">
       <c r="A5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7">
       <c r="A7" s="3" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="30">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" ht="28.5">
       <c r="A8" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="30">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" ht="28.5">
       <c r="A9" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10">
       <c r="A10" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="B10" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C10" s="1"/>
       <c r="E10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11">
       <c r="A11" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B11" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C11" s="1"/>
       <c r="E11" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12">
       <c r="A12" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="B12" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E12" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13">
       <c r="A13" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="B13" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="C13" s="1"/>
       <c r="E13" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E14" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15" ht="34.5" customHeight="1">
+      <c r="A15" t="s">
+        <v>37</v>
+      </c>
+      <c r="B15" t="s">
         <v>38</v>
       </c>
-      <c r="B14" t="s">
-        <v>24</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E14" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="34.5" customHeight="1">
-      <c r="A15" t="s">
+      <c r="C15" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="B15" t="s">
-        <v>27</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>28</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>40</v>
       </c>
       <c r="E15" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>